<commit_message>
feat: 강좌 필터 기능 추가 (course_filter.py)
</commit_message>
<xml_diff>
--- a/데이터/opened_course2024_1.xlsx
+++ b/데이터/opened_course2024_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\AI융개_팀플\데이터\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77147AD7-377D-4239-99E2-04A3168CB5F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DFEF7A-E38B-4AE4-BB17-946779A41E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="심화전공2024_1" sheetId="4" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="409">
   <si>
     <t>수리통계데이터사이언스학부</t>
   </si>
@@ -1256,6 +1256,10 @@
   </si>
   <si>
     <t>서비스디자인공학과</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>바이오식품공학과</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1645,6 +1649,7 @@
   <cols>
     <col min="1" max="1" width="21.3828125" customWidth="1"/>
     <col min="2" max="2" width="27.07421875" customWidth="1"/>
+    <col min="3" max="3" width="18.15234375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -2601,7 +2606,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>211</v>
+        <v>408</v>
       </c>
       <c r="B57" t="s">
         <v>362</v>
@@ -3103,7 +3108,8 @@
   <dimension ref="A1:E184"/>
   <sheetFormatPr defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="17.61328125" customWidth="1"/>
+    <col min="1" max="1" width="27.15234375" customWidth="1"/>
+    <col min="2" max="2" width="31.3828125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">

</xml_diff>